<commit_message>
web: fix ads.txt format, restore real og-image, source hygiene pass
- ads.txt now declares pub-9767914878112531 (was ca-pub-..., wrong
  format per Google's spec, likely suppressing Auto ads matching)
- og-image.png regenerated as a real 1200x630 PNG; fixed the test that
  was silently reverting it to a placeholder stub on every test run
- replaced literal double-hyphens with real em dashes across content
  and rendered pages
- removed manual ad-placeholder markup now superseded by Auto ads
- removed internal task/spec-id references from source comments and
  test titles ahead of the next push
</commit_message>
<xml_diff>
--- a/dist/print/05-tracker-workbook.xlsx
+++ b/dist/print/05-tracker-workbook.xlsx
@@ -43,7 +43,7 @@
     <t xml:space="preserve">This workbook has no macros. Every computed column uses ordinary spreadsheet formulas, so it keeps working if you copy or import it into another spreadsheet application.</t>
   </si>
   <si>
-    <t xml:space="preserve">Not endorsed by or affiliated with Riot Games. League of Legends is a trademark of Riot Games, Inc.</t>
+    <t xml:space="preserve">Solo Queue Practice System was created under Riot Games’ “Legal Jibber Jabber” policy using assets owned by Riot Games. Riot Games does not endorse or sponsor this project. League of Legends is a trademark of Riot Games, Inc.</t>
   </si>
   <si>
     <t xml:space="preserve">v1.0.0 - last reviewed 2026-08-12</t>
@@ -235,7 +235,7 @@
     <t xml:space="preserve">Stretch target:</t>
   </si>
   <si>
-    <t xml:space="preserve">The stricter practice-tool challenge target -- roughly perfect last-hitting with minimal jungle-camp cheats.</t>
+    <t xml:space="preserve">The stricter practice-tool challenge target — roughly perfect last-hitting with minimal jungle-camp cheats.</t>
   </si>
 </sst>
 </file>

</xml_diff>